<commit_message>
server.py and form code
</commit_message>
<xml_diff>
--- a/server/events.xlsx
+++ b/server/events.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,126 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tester description of event space and event itself</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sports &amp; Fitness</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>23:09</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>tester drive</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>55</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>http://image.jpg</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Olamipo Aderibigbe</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>user_1773858004536</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>testttt</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>testttttttttttttttttttttttttttttttttttttt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>23:12</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1263 International Mews</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>55</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>http://image.jpg</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Olamipo Aderibigbe</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>user_1773858004536</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>